<commit_message>
M025 v2.0: mig_307d sensitivity publication outputs (post mig_307c)
Add m025_sensitivity_lib for Wilson CIs on ROM, era-split Sens/Spec/PPV/NPV
with Wilson intervals, per-era ordinal-TR ROC AUC, and matplotlib figures.

Extend build_m025_final_xlsx.py to enrich era/window sensitivity sheets with
lo_95/hi_95 (and window rom_w*_lo/hi), export CSV sidecars and 300 DPI PNGs
under 06_figures_sensitivity/, and refresh M025_tables_and_summary.xlsx.

Add m025_sensitivity_mig_307d.py for idempotent main.signoff_migration insert.

Regenerated package workbooks and artifacts from MotherDuck
thyroid_canonical_publication_v1_0; signoff row mig_307d applied on target DB.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/M025_FINAL_PACKAGE/M025_tables_and_summary.xlsx
+++ b/M025_FINAL_PACKAGE/M025_tables_and_summary.xlsx
@@ -496,7 +496,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Built 2026-05-05T05:08:53.125637+00:00. Manuscript headline = patient-level. Nodule-level = sister analysis.</t>
+          <t>Built 2026-05-05T05:18:12.241134+00:00. Manuscript headline = patient-level. Nodule-level = sister analysis.</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-05-05T05:08:53.125637+00:00</t>
+          <t>2026-05-05T05:18:12.241134+00:00</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>mig_307 (manuscript closeout) + mig_307b (analytic spine refresh)</t>
+          <t>mig_307b (analytic spine) + mig_307c (sensitivity tables) + mig_307d (sensitivity publication outputs)</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Locked from cursor 1d4ecc1 and Cowork pre-bake + mig_307c sensitivity arms.</t>
+          <t>mig_307c sensitivity tables; mig_307d adds Wilson 95% CIs, diagnostics CSVs, and figures under 06_figures_sensitivity/.</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1824,6 +1824,8 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1836,7 +1838,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Era boundary = surg_first_date &lt; 2017-05-01 (ACR TI-RADS 2017 publication date).</t>
+          <t>Era boundary = surg_first_date &lt; 2017-05-01 (ACR TI-RADS 2017 publication date). lo_95 / hi_95 = Wilson 95% CI for ROM (n_malignant / n_total).</t>
         </is>
       </c>
     </row>
@@ -1896,6 +1898,16 @@
           <t>fp_thr5</t>
         </is>
       </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>lo_95</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>hi_95</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1935,6 +1947,12 @@
       <c r="K5" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="L5" s="6" t="n">
+        <v>24.06</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>34.82</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1974,6 +1992,12 @@
       <c r="K6" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="L6" s="6" t="n">
+        <v>25.89</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>37.88</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2013,6 +2037,12 @@
       <c r="K7" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="L7" s="6" t="n">
+        <v>24.86</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>31.31</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2052,6 +2082,12 @@
       <c r="K8" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="L8" s="6" t="n">
+        <v>43.55</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>52.85</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -2090,6 +2126,12 @@
       </c>
       <c r="K9" s="6" t="n">
         <v>534</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>55.35</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>60.77</v>
       </c>
     </row>
     <row r="10">
@@ -2126,6 +2168,12 @@
       <c r="K10" s="6" t="n">
         <v>534</v>
       </c>
+      <c r="L10" s="6" t="n">
+        <v>42.58</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>46.16</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -2165,6 +2213,12 @@
       <c r="K11" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="L11" s="6" t="n">
+        <v>15.99</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>35.96</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -2204,6 +2258,12 @@
       <c r="K12" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="L12" s="6" t="n">
+        <v>23.88</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>45.38</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -2243,6 +2303,12 @@
       <c r="K13" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="L13" s="6" t="n">
+        <v>17.49</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>33.81</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -2282,6 +2348,12 @@
       <c r="K14" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="L14" s="6" t="n">
+        <v>28.16</v>
+      </c>
+      <c r="M14" s="6" t="n">
+        <v>53.93</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -2320,6 +2392,12 @@
       </c>
       <c r="K15" s="6" t="n">
         <v>44</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>72.62</v>
       </c>
     </row>
     <row r="16">
@@ -2355,6 +2433,12 @@
       </c>
       <c r="K16" s="6" t="n">
         <v>44</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>35.48</v>
+      </c>
+      <c r="M16" s="6" t="n">
+        <v>44.79</v>
       </c>
     </row>
   </sheetData>
@@ -2368,7 +2452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2376,6 +2460,8 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2388,7 +2474,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Era boundary = exam_date &lt; 2017-05-01.</t>
+          <t>Era boundary = exam_date &lt; 2017-05-01. lo_95 / hi_95 = Wilson CI for ROM.</t>
         </is>
       </c>
     </row>
@@ -2418,6 +2504,16 @@
           <t>rom_pct</t>
         </is>
       </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>lo_95</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>hi_95</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2439,6 +2535,12 @@
       <c r="E5" s="6" t="n">
         <v>12.9</v>
       </c>
+      <c r="F5" s="6" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>28.85</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2460,6 +2562,12 @@
       <c r="E6" s="6" t="n">
         <v>8.65</v>
       </c>
+      <c r="F6" s="6" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>10.24</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2481,6 +2589,12 @@
       <c r="E7" s="6" t="n">
         <v>18.03</v>
       </c>
+      <c r="F7" s="6" t="n">
+        <v>15.48</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>20.9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2501,6 +2615,12 @@
       </c>
       <c r="E8" s="6" t="n">
         <v>24.37</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>21.94</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>26.98</v>
       </c>
     </row>
     <row r="9">
@@ -2519,6 +2639,12 @@
       <c r="E9" s="6" t="n">
         <v>16.18</v>
       </c>
+      <c r="F9" s="6" t="n">
+        <v>14.97</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>17.48</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -2540,6 +2666,12 @@
       <c r="E10" s="6" t="n">
         <v>13.17</v>
       </c>
+      <c r="F10" s="6" t="n">
+        <v>8.859999999999999</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>19.14</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -2561,6 +2693,12 @@
       <c r="E11" s="6" t="n">
         <v>24.72</v>
       </c>
+      <c r="F11" s="6" t="n">
+        <v>16.93</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>34.6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -2581,6 +2719,12 @@
       </c>
       <c r="E12" s="6" t="n">
         <v>41.6</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>33.34</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>50.37</v>
       </c>
     </row>
     <row r="13">
@@ -2598,6 +2742,12 @@
       </c>
       <c r="E13" s="6" t="n">
         <v>25.2</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>29.79</v>
       </c>
     </row>
   </sheetData>
@@ -2611,7 +2761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2627,6 +2777,14 @@
     <col width="27" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2639,7 +2797,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Recomputes ROM at 365 / 180 / 90 / 30 day windows. Median US-to-malignant-surgery interval ~60–80 days.</t>
+          <t>ROM at 365 / 180 / 90 / 30 d: Wilson 95% CIs in rom_w*_lo_95 / rom_w*_hi_95 vs n_total.</t>
         </is>
       </c>
     </row>
@@ -2709,6 +2867,46 @@
           <t>q95_days_to_surg_malig</t>
         </is>
       </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>rom_w365_lo_95</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>rom_w365_hi_95</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>rom_w180_lo_95</t>
+        </is>
+      </c>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>rom_w180_hi_95</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>rom_w90_lo_95</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>rom_w90_hi_95</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>rom_w30_lo_95</t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>rom_w30_hi_95</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2752,6 +2950,30 @@
       <c r="M5" s="5" t="n">
         <v>56</v>
       </c>
+      <c r="N5" s="6" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>28.85</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="Q5" s="6" t="n">
+        <v>28.85</v>
+      </c>
+      <c r="R5" s="6" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>28.85</v>
+      </c>
+      <c r="T5" s="6" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="U5" s="6" t="n">
+        <v>24.9</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2795,6 +3017,30 @@
       <c r="M6" s="5" t="n">
         <v>288</v>
       </c>
+      <c r="N6" s="6" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="O6" s="6" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="P6" s="6" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="Q6" s="6" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="S6" s="6" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="T6" s="6" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="U6" s="6" t="n">
+        <v>2.97</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2838,6 +3084,30 @@
       <c r="M7" s="5" t="n">
         <v>291</v>
       </c>
+      <c r="N7" s="6" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>21.47</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>13.42</v>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>18.28</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="S7" s="6" t="n">
+        <v>13.57</v>
+      </c>
+      <c r="T7" s="6" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="U7" s="6" t="n">
+        <v>7.84</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2880,6 +3150,30 @@
       </c>
       <c r="M8" s="5" t="n">
         <v>264</v>
+      </c>
+      <c r="N8" s="6" t="n">
+        <v>23.74</v>
+      </c>
+      <c r="O8" s="6" t="n">
+        <v>28.62</v>
+      </c>
+      <c r="P8" s="6" t="n">
+        <v>19.94</v>
+      </c>
+      <c r="Q8" s="6" t="n">
+        <v>24.55</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>14.79</v>
+      </c>
+      <c r="S8" s="6" t="n">
+        <v>18.94</v>
+      </c>
+      <c r="T8" s="6" t="n">
+        <v>7.48</v>
+      </c>
+      <c r="U8" s="6" t="n">
+        <v>10.66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>